<commit_message>
model update and archictecture change
</commit_message>
<xml_diff>
--- a/outputs/scenario_summary.xlsx
+++ b/outputs/scenario_summary.xlsx
@@ -51987,7 +51987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B84"/>
+  <dimension ref="A1:B82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -52761,7 +52761,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>hurdle_completion_trigger.execute_only_if_lp_fully_redeemed</t>
+          <t>backend_liquidity_strategy.enabled</t>
         </is>
       </c>
       <c r="B76" t="b">
@@ -52771,82 +52771,62 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>backend_liquidity_strategy.enabled</t>
-        </is>
-      </c>
-      <c r="B77" t="b">
-        <v>1</v>
+          <t>backend_liquidity_strategy.target_years</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>[5, 7, 10]</t>
+        </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>backend_liquidity_strategy.target_years</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>[5, 7, 10]</t>
-        </is>
+          <t>backend_liquidity_strategy.refi_first</t>
+        </is>
+      </c>
+      <c r="B78" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>backend_liquidity_strategy.refi_first</t>
-        </is>
-      </c>
-      <c r="B79" t="b">
-        <v>1</v>
+          <t>backend_liquidity_strategy.max_refi_pct_of_re_nav</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>0.35</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>backend_liquidity_strategy.max_refi_pct_of_re_nav</t>
+          <t>backend_liquidity_strategy.max_hf_liquidation_pct</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>backend_liquidity_strategy.max_hf_liquidation_pct</t>
-        </is>
-      </c>
-      <c r="B81" t="n">
-        <v>0.5</v>
+          <t>backend_liquidity_strategy.use_retained_cash</t>
+        </is>
+      </c>
+      <c r="B81" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>backend_liquidity_strategy.use_retained_cash</t>
+          <t>backend_liquidity_strategy.use_reserve</t>
         </is>
       </c>
       <c r="B82" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>backend_liquidity_strategy.use_reserve</t>
-        </is>
-      </c>
-      <c r="B83" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>backend_liquidity_strategy.execute_only_if_lp_hurdle_completed</t>
-        </is>
-      </c>
-      <c r="B84" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>